<commit_message>
docs: add income import excel template
Add the actual Excel sample with the required columns: short drama title, channel, income, and date.
</commit_message>
<xml_diff>
--- a/docs/templates/收益导入模板.xlsx
+++ b/docs/templates/收益导入模板.xlsx
@@ -14,18 +14,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>剧目ID</t>
-  </si>
-  <si>
-    <t>日期(YYYY-MM-DD)</t>
-  </si>
-  <si>
-    <t>收入金额(元)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+  <si>
+    <t>短剧名称</t>
+  </si>
+  <si>
+    <t>渠道</t>
+  </si>
+  <si>
+    <t>收益</t>
+  </si>
+  <si>
+    <t>日期</t>
+  </si>
+  <si>
+    <t>总裁的逆袭新娘</t>
+  </si>
+  <si>
+    <t>抖音</t>
   </si>
   <si>
     <t>2026-05-26</t>
+  </si>
+  <si>
+    <t>快手</t>
   </si>
   <si>
     <t>2026-05-27</t>
@@ -335,7 +347,8 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="3" min="1" width="20"/>
+    <col customWidth="true" max="1" min="1" width="28"/>
+    <col customWidth="true" max="4" min="2" width="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -348,27 +361,36 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C2">
         <v>123.45</v>
       </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>1</v>
+      <c r="A3" t="s">
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C3">
         <v>88</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>